<commit_message>
Un seul modèle de fichier banque (Banque.xlsx) : les autres modèles sont retirés
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8s2z31P3cgDQRDppUofdK
</commit_message>
<xml_diff>
--- a/Imports/modeles/Lexique.xlsx
+++ b/Imports/modeles/Lexique.xlsx
@@ -648,7 +648,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tiers : membres, fournisseurs…</t>
+          <t>Tiers : clients, fournisseurs…</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Compte | Type | Nom | Prénom | Adresse | Code postal | Ville | Téléphone | E-mail | Date d'adhésion | Statut | Cotisation annuelle</t>
+          <t>Compte | Type | Nom | Prénom | Adresse | Code postal | Ville | Téléphone | E-mail</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Membre (par défaut), Fournisseur…</t>
+          <t>Client (par défaut), Fournisseur…</t>
         </is>
       </c>
     </row>
@@ -1608,81 +1608,93 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tiers.xlsx</t>
+          <t>Traductions.xlsx</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Date d'adhésion</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>Opération (hébreu)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>date jj/mm/aaaa</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Membres</t>
+          <t>Libellé du relevé bancaire</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tiers.xlsx</t>
+          <t>Traductions.xlsx</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Statut</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>Traduction</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Actif / Honoraire / Démissionnaire</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Membres</t>
+          <t>Traduction française</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Tiers.xlsx</t>
+          <t>Budget.xlsx</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cotisation annuelle</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
+          <t>Exercice</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>montant (nombre, sans symbole)</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Cotisation attendue</t>
+          <t>Libellé de l'exercice (Exercices.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Traductions.xlsx</t>
+          <t>Budget.xlsx</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Opération (hébreu)</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1692,39 +1704,31 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>texte</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Libellé du relevé bancaire</t>
-        </is>
-      </c>
+          <t>Charges / Produits</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Traductions.xlsx</t>
+          <t>Budget.xlsx</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Traduction</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Compte</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>code (texte)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Traduction française</t>
+          <t>Cible : un compte…</t>
         </is>
       </c>
     </row>
@@ -1736,22 +1740,18 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Exercice</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Anal</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>code (texte)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Libellé de l'exercice (Exercices.xlsx)</t>
+          <t>… ou un code Anal (une seule cible)</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Montant</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1773,46 +1773,58 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Charges / Produits</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr"/>
+          <t>montant (nombre, sans symbole)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Montant budgété</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Budget.xlsx</t>
+          <t>Ecritures.xlsx</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Compte</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+          <t>Mvt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>entier</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Cible : un compte…</t>
+          <t>N° de mouvement (une opération équilibrée)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Budget.xlsx</t>
+          <t>Ecritures.xlsx</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Anal</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+          <t>Jnl</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>code (texte)</t>
@@ -1820,19 +1832,19 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>… ou un code Anal (une seule cible)</t>
+          <t>Journal (Journaux.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Budget.xlsx</t>
+          <t>Ecritures.xlsx</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Montant</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1842,12 +1854,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>montant (nombre, sans symbole)</t>
+          <t>date jj/mm/aaaa</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Montant budgété</t>
+          <t>Même date sur toutes les lignes du Mvt</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1871,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mvt</t>
+          <t>Compte</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1869,12 +1881,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>entier</t>
+          <t>code (texte)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>N° de mouvement (une opération équilibrée)</t>
+          <t>Compte (PlanComptable.xlsx)</t>
         </is>
       </c>
     </row>
@@ -1886,22 +1898,18 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Jnl</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>LibelCompte</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Journal (Journaux.xlsx)</t>
+          <t>Rappel du plan, non lu</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1921,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Libelle</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1923,14 +1931,10 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>date jj/mm/aaaa</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Même date sur toutes les lignes du Mvt</t>
-        </is>
-      </c>
+          <t>texte</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1940,22 +1944,18 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Compte</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>montant (nombre, sans symbole)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Compte (PlanComptable.xlsx)</t>
+          <t>Débit OU crédit</t>
         </is>
       </c>
     </row>
@@ -1967,18 +1967,18 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LibelCompte</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>montant (nombre, sans symbole)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Rappel du plan, non lu</t>
+          <t>Débit OU crédit</t>
         </is>
       </c>
     </row>
@@ -1990,20 +1990,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Libelle</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Anal</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>texte</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
+          <t>code (texte)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Rappel du plan (code Anal du compte) : le plan fait foi</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2013,18 +2013,18 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Debit</t>
+          <t>LibelAnal</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>montant (nombre, sans symbole)</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Débit OU crédit</t>
+          <t>Rappel, non lu</t>
         </is>
       </c>
     </row>
@@ -2036,18 +2036,18 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Credit</t>
+          <t>Lien</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>montant (nombre, sans symbole)</t>
+          <t>adresse https://</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Débit OU crédit</t>
+          <t>Document justificatif en ligne, joint au Mvt</t>
         </is>
       </c>
     </row>
@@ -2059,87 +2059,99 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Anal</t>
+          <t>Let</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>3 lettres majuscules</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Rappel du plan (code Anal du compte) : le plan fait foi</t>
+          <t>Code de lettrage (AAA, AAB…), vide hors comptes de tiers</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ecritures.xlsx</t>
+          <t>Libelles.xlsx</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LibelAnal</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
+          <t>Mvt</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>entier</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Rappel, non lu</t>
+          <t>N° de mouvement (une opération équilibrée)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ecritures.xlsx</t>
+          <t>Libelles.xlsx</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Lien</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr"/>
+          <t>Jnl</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>adresse https://</t>
+          <t>code (texte)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Document justificatif en ligne, joint au Mvt</t>
+          <t>Journal (Journaux.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ecritures.xlsx</t>
+          <t>Libelles.xlsx</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Let</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>3 lettres majuscules</t>
+          <t>date jj/mm/aaaa</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Code de lettrage (AAA, AAB…), vide hors comptes de tiers</t>
+          <t>Même date sur toutes les lignes du Mvt</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2163,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Mvt</t>
+          <t>Compte</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2161,12 +2173,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>entier</t>
+          <t>code (texte)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>N° de mouvement (une opération équilibrée)</t>
+          <t>Compte (PlanComptable.xlsx)</t>
         </is>
       </c>
     </row>
@@ -2178,22 +2190,18 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Jnl</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>LibelCompte</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Journal (Journaux.xlsx)</t>
+          <t>Rappel du plan, non lu</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2213,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Libelle</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2215,14 +2223,10 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>date jj/mm/aaaa</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Même date sur toutes les lignes du Mvt</t>
-        </is>
-      </c>
+          <t>texte</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2232,22 +2236,18 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Compte</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>montant (nombre, sans symbole)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Compte (PlanComptable.xlsx)</t>
+          <t>Débit OU crédit</t>
         </is>
       </c>
     </row>
@@ -2259,18 +2259,18 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LibelCompte</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>montant (nombre, sans symbole)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Rappel du plan, non lu</t>
+          <t>Débit OU crédit</t>
         </is>
       </c>
     </row>
@@ -2282,20 +2282,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Libelle</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Anal</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>texte</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
+          <t>code (texte)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Rappel du plan (code Anal du compte) : le plan fait foi</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2305,18 +2305,18 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Debit</t>
+          <t>LibelAnal</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>montant (nombre, sans symbole)</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Débit OU crédit</t>
+          <t>Rappel, non lu</t>
         </is>
       </c>
     </row>
@@ -2328,18 +2328,18 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Credit</t>
+          <t>Lien</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>montant (nombre, sans symbole)</t>
+          <t>adresse https://</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Débit OU crédit</t>
+          <t>Document justificatif en ligne, joint au Mvt</t>
         </is>
       </c>
     </row>
@@ -2351,48 +2351,52 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Anal</t>
+          <t>Let</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>3 lettres majuscules</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Rappel du plan (code Anal du compte) : le plan fait foi</t>
+          <t>Code de lettrage (AAA, AAB…), vide hors comptes de tiers</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Libelles.xlsx</t>
+          <t>Liens.xlsx</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LibelAnal</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
+          <t>Mvt</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>entier</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Rappel, non lu</t>
+          <t>N° du mouvement (Ecritures.xlsx ou site)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Libelles.xlsx</t>
+          <t>Liens.xlsx</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2400,7 +2404,11 @@
           <t>Lien</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
           <t>adresse https://</t>
@@ -2408,42 +2416,42 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Document justificatif en ligne, joint au Mvt</t>
+          <t>Lien du document</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Libelles.xlsx</t>
+          <t>Liens.xlsx</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Let</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>3 lettres majuscules</t>
+          <t>texte</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Code de lettrage (AAA, AAB…), vide hors comptes de tiers</t>
+          <t>Tiers, catégorie…</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Liens.xlsx</t>
+          <t>Banque.xlsx</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Mvt</t>
+          <t>Jnl</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2453,24 +2461,24 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>entier</t>
+          <t>code (texte)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>N° du mouvement (Ecritures.xlsx ou site)</t>
+          <t>Journal de la banque ou de la caisse (Journaux)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Liens.xlsx</t>
+          <t>Banque.xlsx</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Lien</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2480,27 +2488,27 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>adresse https://</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Lien du document</t>
-        </is>
-      </c>
+          <t>date jj/mm/aaaa</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Liens.xlsx</t>
+          <t>Banque.xlsx</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
+          <t>Libelle</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr">
         <is>
           <t>texte</t>
@@ -2508,7 +2516,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Tiers, catégorie…</t>
+          <t>Libellé de la banque, tel quel (hébreu conservé)</t>
         </is>
       </c>
     </row>
@@ -2520,22 +2528,18 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Jnl</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>code (texte)</t>
+          <t>montant (nombre, sans symbole)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Journal de la banque ou de la caisse (Journaux)</t>
+          <t>Entrée : Debit OU Credit (l'autre colonne vide ou à 0)</t>
         </is>
       </c>
     </row>
@@ -2547,20 +2551,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>date jj/mm/aaaa</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr"/>
+          <t>montant (nombre, sans symbole)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Sortie : Debit OU Credit</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2570,89 +2574,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Libelle</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+          <t>Solde</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
-          <t>texte</t>
+          <t>montant (nombre, sans symbole)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
-        <is>
-          <t>Libellé de la banque, tel quel (hébreu conservé)</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Banque.xlsx</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>montant (nombre, sans symbole)</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Entrée : Debit OU Credit (l'autre colonne vide ou à 0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Banque.xlsx</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>montant (nombre, sans symbole)</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Sortie : Debit OU Credit</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Banque.xlsx</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Solde</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>montant (nombre, sans symbole)</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
         <is>
           <t>Solde après la ligne, si la banque le donne (Bit n'en donne pas) ; sert à contrôler le relevé</t>
         </is>

</xml_diff>